<commit_message>
all files for now
</commit_message>
<xml_diff>
--- a/Documentation/docs/Product Book/PPIQ_Backlog_v2_9_1_03Aug2026.xlsx
+++ b/Documentation/docs/Product Book/PPIQ_Backlog_v2_9_1_03Aug2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\PlantProcess-IQ\Documentation\docs\Product Book\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0F014AA-4272-43FA-9F3C-50DD12563623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EB4BBDE-2C52-44DD-843B-BD99CB96710D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="394" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2658,7 +2658,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2706,9 +2706,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2724,6 +2721,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3037,8 +3040,8 @@
     <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="175.140625" style="23" customWidth="1"/>
-    <col min="9" max="9" width="136.5703125" style="27" customWidth="1"/>
+    <col min="8" max="8" width="175.140625" style="22" customWidth="1"/>
+    <col min="9" max="9" width="136.5703125" style="26" customWidth="1"/>
     <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -3065,7 +3068,7 @@
       <c r="G1" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="22" t="s">
+      <c r="H1" s="21" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="17" t="s">
@@ -3100,10 +3103,10 @@
       <c r="G2" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="24" t="s">
+      <c r="H2" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="24" t="s">
+      <c r="I2" s="23" t="s">
         <v>19</v>
       </c>
       <c r="J2" s="18">
@@ -3135,10 +3138,10 @@
       <c r="G3" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="24" t="s">
+      <c r="I3" s="23" t="s">
         <v>25</v>
       </c>
       <c r="J3" s="18">
@@ -3170,10 +3173,10 @@
       <c r="G4" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="24" t="s">
+      <c r="H4" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="24" t="s">
+      <c r="I4" s="23" t="s">
         <v>31</v>
       </c>
       <c r="J4" s="18">
@@ -3205,10 +3208,10 @@
       <c r="G5" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="H5" s="24" t="s">
+      <c r="H5" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="I5" s="24" t="s">
+      <c r="I5" s="23" t="s">
         <v>37</v>
       </c>
       <c r="J5" s="18">
@@ -3240,10 +3243,10 @@
       <c r="G6" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="24" t="s">
+      <c r="H6" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="I6" s="24" t="s">
+      <c r="I6" s="23" t="s">
         <v>43</v>
       </c>
       <c r="J6" s="18">
@@ -3275,10 +3278,10 @@
       <c r="G7" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="24" t="s">
+      <c r="H7" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="I7" s="24" t="s">
+      <c r="I7" s="23" t="s">
         <v>47</v>
       </c>
       <c r="J7" s="18">
@@ -3310,10 +3313,10 @@
       <c r="G8" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="I8" s="24" t="s">
+      <c r="I8" s="23" t="s">
         <v>51</v>
       </c>
       <c r="J8" s="18">
@@ -3345,10 +3348,10 @@
       <c r="G9" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="24" t="s">
+      <c r="H9" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="I9" s="24" t="s">
+      <c r="I9" s="23" t="s">
         <v>57</v>
       </c>
       <c r="J9" s="18">
@@ -3380,10 +3383,10 @@
       <c r="G10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="24" t="s">
+      <c r="H10" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="I10" s="24" t="s">
+      <c r="I10" s="23" t="s">
         <v>63</v>
       </c>
       <c r="J10" s="18">
@@ -3415,10 +3418,10 @@
       <c r="G11" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="24" t="s">
+      <c r="H11" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="I11" s="24" t="s">
+      <c r="I11" s="23" t="s">
         <v>68</v>
       </c>
       <c r="J11" s="18">
@@ -3450,10 +3453,10 @@
       <c r="G12" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="H12" s="24" t="s">
+      <c r="H12" s="23" t="s">
         <v>73</v>
       </c>
-      <c r="I12" s="24" t="s">
+      <c r="I12" s="23" t="s">
         <v>74</v>
       </c>
       <c r="J12" s="18">
@@ -3485,10 +3488,10 @@
       <c r="G13" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="24" t="s">
+      <c r="H13" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="I13" s="24" t="s">
+      <c r="I13" s="23" t="s">
         <v>79</v>
       </c>
       <c r="J13" s="18">
@@ -3520,10 +3523,10 @@
       <c r="G14" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="24" t="s">
+      <c r="H14" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="I14" s="24" t="s">
+      <c r="I14" s="23" t="s">
         <v>85</v>
       </c>
       <c r="J14" s="18">
@@ -3555,10 +3558,10 @@
       <c r="G15" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H15" s="24" t="s">
+      <c r="H15" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="I15" s="24" t="s">
+      <c r="I15" s="23" t="s">
         <v>89</v>
       </c>
       <c r="J15" s="18">
@@ -3590,10 +3593,10 @@
       <c r="G16" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H16" s="24" t="s">
+      <c r="H16" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="I16" s="24" t="s">
+      <c r="I16" s="23" t="s">
         <v>94</v>
       </c>
       <c r="J16" s="18">
@@ -3625,10 +3628,10 @@
       <c r="G17" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H17" s="24" t="s">
+      <c r="H17" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="24" t="s">
+      <c r="I17" s="23" t="s">
         <v>98</v>
       </c>
       <c r="J17" s="18">
@@ -3660,10 +3663,10 @@
       <c r="G18" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H18" s="24" t="s">
+      <c r="H18" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="I18" s="24" t="s">
+      <c r="I18" s="23" t="s">
         <v>102</v>
       </c>
       <c r="J18" s="18">
@@ -3695,10 +3698,10 @@
       <c r="G19" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H19" s="24" t="s">
+      <c r="H19" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="I19" s="24" t="s">
+      <c r="I19" s="23" t="s">
         <v>106</v>
       </c>
       <c r="J19" s="18">
@@ -3730,10 +3733,10 @@
       <c r="G20" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="H20" s="24" t="s">
+      <c r="H20" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="I20" s="24" t="s">
+      <c r="I20" s="23" t="s">
         <v>110</v>
       </c>
       <c r="J20" s="18">
@@ -3765,10 +3768,10 @@
       <c r="G21" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="H21" s="24" t="s">
+      <c r="H21" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="I21" s="24" t="s">
+      <c r="I21" s="23" t="s">
         <v>114</v>
       </c>
       <c r="J21" s="18">
@@ -3800,10 +3803,10 @@
       <c r="G22" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="H22" s="24" t="s">
+      <c r="H22" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="I22" s="24" t="s">
+      <c r="I22" s="23" t="s">
         <v>118</v>
       </c>
       <c r="J22" s="18">
@@ -3835,10 +3838,10 @@
       <c r="G23" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H23" s="24" t="s">
+      <c r="H23" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="I23" s="24" t="s">
+      <c r="I23" s="23" t="s">
         <v>122</v>
       </c>
       <c r="J23" s="18">
@@ -3870,10 +3873,10 @@
       <c r="G24" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H24" s="24" t="s">
+      <c r="H24" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="I24" s="24" t="s">
+      <c r="I24" s="23" t="s">
         <v>126</v>
       </c>
       <c r="J24" s="18">
@@ -3905,10 +3908,10 @@
       <c r="G25" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H25" s="24" t="s">
+      <c r="H25" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="I25" s="24" t="s">
+      <c r="I25" s="23" t="s">
         <v>130</v>
       </c>
       <c r="J25" s="18">
@@ -3940,10 +3943,10 @@
       <c r="G26" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H26" s="24" t="s">
+      <c r="H26" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="I26" s="24" t="s">
+      <c r="I26" s="23" t="s">
         <v>135</v>
       </c>
       <c r="J26" s="18">
@@ -3954,38 +3957,38 @@
       </c>
     </row>
     <row r="27" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="B27" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C27" s="19" t="s">
+      <c r="B27" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="D27" s="19" t="s">
+      <c r="D27" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="E27" s="19" t="s">
+      <c r="E27" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="F27" s="19" t="s">
+      <c r="F27" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="G27" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="H27" s="25" t="s">
+      <c r="G27" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H27" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="I27" s="25" t="s">
+      <c r="I27" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="J27" s="19">
+      <c r="J27" s="18">
         <v>6</v>
       </c>
-      <c r="K27" s="19" t="s">
-        <v>90</v>
+      <c r="K27" s="18" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="75" x14ac:dyDescent="0.25">
@@ -4010,10 +4013,10 @@
       <c r="G28" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H28" s="25" t="s">
+      <c r="H28" s="24" t="s">
         <v>142</v>
       </c>
-      <c r="I28" s="25" t="s">
+      <c r="I28" s="24" t="s">
         <v>143</v>
       </c>
       <c r="J28" s="19">
@@ -4045,10 +4048,10 @@
       <c r="G29" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H29" s="25" t="s">
+      <c r="H29" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="I29" s="25" t="s">
+      <c r="I29" s="24" t="s">
         <v>147</v>
       </c>
       <c r="J29" s="19">
@@ -4080,10 +4083,10 @@
       <c r="G30" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H30" s="25" t="s">
+      <c r="H30" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="I30" s="25" t="s">
+      <c r="I30" s="24" t="s">
         <v>151</v>
       </c>
       <c r="J30" s="19">
@@ -4115,10 +4118,10 @@
       <c r="G31" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H31" s="25" t="s">
+      <c r="H31" s="24" t="s">
         <v>155</v>
       </c>
-      <c r="I31" s="25" t="s">
+      <c r="I31" s="24" t="s">
         <v>156</v>
       </c>
       <c r="J31" s="19">
@@ -4150,10 +4153,10 @@
       <c r="G32" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H32" s="25" t="s">
+      <c r="H32" s="24" t="s">
         <v>159</v>
       </c>
-      <c r="I32" s="25" t="s">
+      <c r="I32" s="24" t="s">
         <v>160</v>
       </c>
       <c r="J32" s="19">
@@ -4163,7 +4166,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="1:11" s="21" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" s="27" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A33" s="20" t="s">
         <v>161</v>
       </c>
@@ -4185,13 +4188,13 @@
       <c r="G33" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="H33" s="26" t="s">
+      <c r="H33" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="I33" s="26" t="s">
+      <c r="I33" s="25" t="s">
         <v>165</v>
       </c>
-      <c r="J33" s="20">
+      <c r="J33" s="28">
         <v>12</v>
       </c>
       <c r="K33" s="20" t="s">
@@ -4199,73 +4202,73 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A34" s="19" t="s">
+      <c r="A34" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="B34" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C34" s="19" t="s">
+      <c r="B34" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="D34" s="19" t="s">
+      <c r="D34" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="E34" s="19" t="s">
+      <c r="E34" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F34" s="19" t="s">
+      <c r="F34" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="G34" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="H34" s="25" t="s">
+      <c r="G34" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H34" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="I34" s="25" t="s">
+      <c r="I34" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="J34" s="19">
-        <v>12</v>
-      </c>
-      <c r="K34" s="19" t="s">
-        <v>90</v>
+      <c r="J34" s="18">
+        <v>12</v>
+      </c>
+      <c r="K34" s="20" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="B35" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C35" s="19" t="s">
+      <c r="B35" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="D35" s="19" t="s">
+      <c r="D35" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="E35" s="19" t="s">
+      <c r="E35" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F35" s="19" t="s">
+      <c r="F35" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="G35" s="19" t="s">
+      <c r="G35" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="H35" s="25" t="s">
+      <c r="H35" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="I35" s="25" t="s">
+      <c r="I35" s="23" t="s">
         <v>173</v>
       </c>
-      <c r="J35" s="19">
+      <c r="J35" s="18">
         <v>10</v>
       </c>
-      <c r="K35" s="19" t="s">
-        <v>90</v>
+      <c r="K35" s="20" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -4290,10 +4293,10 @@
       <c r="G36" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H36" s="25" t="s">
+      <c r="H36" s="24" t="s">
         <v>177</v>
       </c>
-      <c r="I36" s="25" t="s">
+      <c r="I36" s="24" t="s">
         <v>178</v>
       </c>
       <c r="J36" s="19">
@@ -4325,10 +4328,10 @@
       <c r="G37" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H37" s="25" t="s">
+      <c r="H37" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="I37" s="25" t="s">
+      <c r="I37" s="24" t="s">
         <v>182</v>
       </c>
       <c r="J37" s="19">
@@ -4360,10 +4363,10 @@
       <c r="G38" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="H38" s="25" t="s">
+      <c r="H38" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="I38" s="25" t="s">
+      <c r="I38" s="24" t="s">
         <v>186</v>
       </c>
       <c r="J38" s="19">
@@ -4395,10 +4398,10 @@
       <c r="G39" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H39" s="25" t="s">
+      <c r="H39" s="24" t="s">
         <v>189</v>
       </c>
-      <c r="I39" s="25" t="s">
+      <c r="I39" s="24" t="s">
         <v>190</v>
       </c>
       <c r="J39" s="19">
@@ -4430,10 +4433,10 @@
       <c r="G40" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H40" s="25" t="s">
+      <c r="H40" s="24" t="s">
         <v>194</v>
       </c>
-      <c r="I40" s="25" t="s">
+      <c r="I40" s="24" t="s">
         <v>195</v>
       </c>
       <c r="J40" s="19">
@@ -4465,10 +4468,10 @@
       <c r="G41" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H41" s="25" t="s">
+      <c r="H41" s="24" t="s">
         <v>198</v>
       </c>
-      <c r="I41" s="25" t="s">
+      <c r="I41" s="24" t="s">
         <v>199</v>
       </c>
       <c r="J41" s="19">
@@ -4500,10 +4503,10 @@
       <c r="G42" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H42" s="25" t="s">
+      <c r="H42" s="24" t="s">
         <v>203</v>
       </c>
-      <c r="I42" s="25" t="s">
+      <c r="I42" s="24" t="s">
         <v>204</v>
       </c>
       <c r="J42" s="19">
@@ -4535,10 +4538,10 @@
       <c r="G43" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H43" s="25" t="s">
+      <c r="H43" s="24" t="s">
         <v>207</v>
       </c>
-      <c r="I43" s="25" t="s">
+      <c r="I43" s="24" t="s">
         <v>208</v>
       </c>
       <c r="J43" s="19">
@@ -4570,10 +4573,10 @@
       <c r="G44" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H44" s="25" t="s">
+      <c r="H44" s="24" t="s">
         <v>211</v>
       </c>
-      <c r="I44" s="25" t="s">
+      <c r="I44" s="24" t="s">
         <v>212</v>
       </c>
       <c r="J44" s="19">
@@ -4605,10 +4608,10 @@
       <c r="G45" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H45" s="25" t="s">
+      <c r="H45" s="24" t="s">
         <v>215</v>
       </c>
-      <c r="I45" s="25" t="s">
+      <c r="I45" s="24" t="s">
         <v>216</v>
       </c>
       <c r="J45" s="19">
@@ -4640,10 +4643,10 @@
       <c r="G46" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H46" s="25" t="s">
+      <c r="H46" s="24" t="s">
         <v>219</v>
       </c>
-      <c r="I46" s="25" t="s">
+      <c r="I46" s="24" t="s">
         <v>220</v>
       </c>
       <c r="J46" s="19">
@@ -4675,10 +4678,10 @@
       <c r="G47" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H47" s="25" t="s">
+      <c r="H47" s="24" t="s">
         <v>224</v>
       </c>
-      <c r="I47" s="25" t="s">
+      <c r="I47" s="24" t="s">
         <v>225</v>
       </c>
       <c r="J47" s="19">
@@ -4710,10 +4713,10 @@
       <c r="G48" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H48" s="25" t="s">
+      <c r="H48" s="24" t="s">
         <v>228</v>
       </c>
-      <c r="I48" s="25" t="s">
+      <c r="I48" s="24" t="s">
         <v>229</v>
       </c>
       <c r="J48" s="19">
@@ -4745,10 +4748,10 @@
       <c r="G49" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H49" s="25" t="s">
+      <c r="H49" s="24" t="s">
         <v>232</v>
       </c>
-      <c r="I49" s="25" t="s">
+      <c r="I49" s="24" t="s">
         <v>233</v>
       </c>
       <c r="J49" s="19">
@@ -4780,10 +4783,10 @@
       <c r="G50" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="H50" s="25" t="s">
+      <c r="H50" s="24" t="s">
         <v>236</v>
       </c>
-      <c r="I50" s="25" t="s">
+      <c r="I50" s="24" t="s">
         <v>237</v>
       </c>
       <c r="J50" s="19">
@@ -4815,10 +4818,10 @@
       <c r="G51" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H51" s="25" t="s">
+      <c r="H51" s="24" t="s">
         <v>240</v>
       </c>
-      <c r="I51" s="25" t="s">
+      <c r="I51" s="24" t="s">
         <v>241</v>
       </c>
       <c r="J51" s="19">
@@ -4850,10 +4853,10 @@
       <c r="G52" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H52" s="25" t="s">
+      <c r="H52" s="24" t="s">
         <v>244</v>
       </c>
-      <c r="I52" s="25" t="s">
+      <c r="I52" s="24" t="s">
         <v>245</v>
       </c>
       <c r="J52" s="19">
@@ -4885,10 +4888,10 @@
       <c r="G53" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H53" s="25" t="s">
+      <c r="H53" s="24" t="s">
         <v>248</v>
       </c>
-      <c r="I53" s="25" t="s">
+      <c r="I53" s="24" t="s">
         <v>249</v>
       </c>
       <c r="J53" s="19">
@@ -4920,10 +4923,10 @@
       <c r="G54" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H54" s="25" t="s">
+      <c r="H54" s="24" t="s">
         <v>253</v>
       </c>
-      <c r="I54" s="25" t="s">
+      <c r="I54" s="24" t="s">
         <v>254</v>
       </c>
       <c r="J54" s="19">
@@ -4955,10 +4958,10 @@
       <c r="G55" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H55" s="25" t="s">
+      <c r="H55" s="24" t="s">
         <v>258</v>
       </c>
-      <c r="I55" s="25" t="s">
+      <c r="I55" s="24" t="s">
         <v>259</v>
       </c>
       <c r="J55" s="19">
@@ -4990,10 +4993,10 @@
       <c r="G56" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H56" s="25" t="s">
+      <c r="H56" s="24" t="s">
         <v>263</v>
       </c>
-      <c r="I56" s="25" t="s">
+      <c r="I56" s="24" t="s">
         <v>264</v>
       </c>
       <c r="J56" s="19">
@@ -5025,10 +5028,10 @@
       <c r="G57" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="H57" s="25" t="s">
+      <c r="H57" s="24" t="s">
         <v>267</v>
       </c>
-      <c r="I57" s="25" t="s">
+      <c r="I57" s="24" t="s">
         <v>268</v>
       </c>
       <c r="J57" s="19">
@@ -5060,10 +5063,10 @@
       <c r="G58" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H58" s="25" t="s">
+      <c r="H58" s="24" t="s">
         <v>272</v>
       </c>
-      <c r="I58" s="25" t="s">
+      <c r="I58" s="24" t="s">
         <v>273</v>
       </c>
       <c r="J58" s="19">
@@ -5095,10 +5098,10 @@
       <c r="G59" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H59" s="25" t="s">
+      <c r="H59" s="24" t="s">
         <v>276</v>
       </c>
-      <c r="I59" s="25" t="s">
+      <c r="I59" s="24" t="s">
         <v>277</v>
       </c>
       <c r="J59" s="19">
@@ -5130,10 +5133,10 @@
       <c r="G60" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H60" s="25" t="s">
+      <c r="H60" s="24" t="s">
         <v>280</v>
       </c>
-      <c r="I60" s="25" t="s">
+      <c r="I60" s="24" t="s">
         <v>281</v>
       </c>
       <c r="J60" s="19">
@@ -5165,10 +5168,10 @@
       <c r="G61" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H61" s="25" t="s">
+      <c r="H61" s="24" t="s">
         <v>284</v>
       </c>
-      <c r="I61" s="25" t="s">
+      <c r="I61" s="24" t="s">
         <v>285</v>
       </c>
       <c r="J61" s="19">
@@ -5200,10 +5203,10 @@
       <c r="G62" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H62" s="25" t="s">
+      <c r="H62" s="24" t="s">
         <v>289</v>
       </c>
-      <c r="I62" s="25" t="s">
+      <c r="I62" s="24" t="s">
         <v>290</v>
       </c>
       <c r="J62" s="19">
@@ -5235,10 +5238,10 @@
       <c r="G63" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H63" s="25" t="s">
+      <c r="H63" s="24" t="s">
         <v>293</v>
       </c>
-      <c r="I63" s="25" t="s">
+      <c r="I63" s="24" t="s">
         <v>294</v>
       </c>
       <c r="J63" s="19">
@@ -5270,10 +5273,10 @@
       <c r="G64" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H64" s="25" t="s">
+      <c r="H64" s="24" t="s">
         <v>298</v>
       </c>
-      <c r="I64" s="25" t="s">
+      <c r="I64" s="24" t="s">
         <v>299</v>
       </c>
       <c r="J64" s="19">
@@ -5305,10 +5308,10 @@
       <c r="G65" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H65" s="25" t="s">
+      <c r="H65" s="24" t="s">
         <v>303</v>
       </c>
-      <c r="I65" s="25" t="s">
+      <c r="I65" s="24" t="s">
         <v>304</v>
       </c>
       <c r="J65" s="19">
@@ -5340,10 +5343,10 @@
       <c r="G66" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H66" s="25" t="s">
+      <c r="H66" s="24" t="s">
         <v>307</v>
       </c>
-      <c r="I66" s="25" t="s">
+      <c r="I66" s="24" t="s">
         <v>308</v>
       </c>
       <c r="J66" s="19">
@@ -5375,10 +5378,10 @@
       <c r="G67" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H67" s="25" t="s">
+      <c r="H67" s="24" t="s">
         <v>311</v>
       </c>
-      <c r="I67" s="25" t="s">
+      <c r="I67" s="24" t="s">
         <v>312</v>
       </c>
       <c r="J67" s="19">
@@ -5410,10 +5413,10 @@
       <c r="G68" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H68" s="25" t="s">
+      <c r="H68" s="24" t="s">
         <v>315</v>
       </c>
-      <c r="I68" s="25" t="s">
+      <c r="I68" s="24" t="s">
         <v>316</v>
       </c>
       <c r="J68" s="19">
@@ -5445,10 +5448,10 @@
       <c r="G69" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H69" s="25" t="s">
+      <c r="H69" s="24" t="s">
         <v>319</v>
       </c>
-      <c r="I69" s="25" t="s">
+      <c r="I69" s="24" t="s">
         <v>320</v>
       </c>
       <c r="J69" s="19">
@@ -5480,10 +5483,10 @@
       <c r="G70" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H70" s="25" t="s">
+      <c r="H70" s="24" t="s">
         <v>326</v>
       </c>
-      <c r="I70" s="25" t="s">
+      <c r="I70" s="24" t="s">
         <v>327</v>
       </c>
       <c r="J70" s="19">
@@ -5515,10 +5518,10 @@
       <c r="G71" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="H71" s="25" t="s">
+      <c r="H71" s="24" t="s">
         <v>330</v>
       </c>
-      <c r="I71" s="25" t="s">
+      <c r="I71" s="24" t="s">
         <v>331</v>
       </c>
       <c r="J71" s="19">
@@ -5550,10 +5553,10 @@
       <c r="G72" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H72" s="25" t="s">
+      <c r="H72" s="24" t="s">
         <v>335</v>
       </c>
-      <c r="I72" s="25" t="s">
+      <c r="I72" s="24" t="s">
         <v>336</v>
       </c>
       <c r="J72" s="19">
@@ -5585,10 +5588,10 @@
       <c r="G73" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H73" s="25" t="s">
+      <c r="H73" s="24" t="s">
         <v>339</v>
       </c>
-      <c r="I73" s="25" t="s">
+      <c r="I73" s="24" t="s">
         <v>340</v>
       </c>
       <c r="J73" s="19">
@@ -5620,10 +5623,10 @@
       <c r="G74" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H74" s="25" t="s">
+      <c r="H74" s="24" t="s">
         <v>344</v>
       </c>
-      <c r="I74" s="25" t="s">
+      <c r="I74" s="24" t="s">
         <v>345</v>
       </c>
       <c r="J74" s="19">
@@ -5655,10 +5658,10 @@
       <c r="G75" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H75" s="25" t="s">
+      <c r="H75" s="24" t="s">
         <v>348</v>
       </c>
-      <c r="I75" s="25" t="s">
+      <c r="I75" s="24" t="s">
         <v>349</v>
       </c>
       <c r="J75" s="19">
@@ -5690,10 +5693,10 @@
       <c r="G76" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H76" s="25" t="s">
+      <c r="H76" s="24" t="s">
         <v>352</v>
       </c>
-      <c r="I76" s="25" t="s">
+      <c r="I76" s="24" t="s">
         <v>353</v>
       </c>
       <c r="J76" s="19">
@@ -5725,10 +5728,10 @@
       <c r="G77" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H77" s="25" t="s">
+      <c r="H77" s="24" t="s">
         <v>356</v>
       </c>
-      <c r="I77" s="25" t="s">
+      <c r="I77" s="24" t="s">
         <v>357</v>
       </c>
       <c r="J77" s="19">
@@ -5760,10 +5763,10 @@
       <c r="G78" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H78" s="25" t="s">
+      <c r="H78" s="24" t="s">
         <v>361</v>
       </c>
-      <c r="I78" s="25" t="s">
+      <c r="I78" s="24" t="s">
         <v>362</v>
       </c>
       <c r="J78" s="19">
@@ -5795,10 +5798,10 @@
       <c r="G79" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H79" s="25" t="s">
+      <c r="H79" s="24" t="s">
         <v>366</v>
       </c>
-      <c r="I79" s="25" t="s">
+      <c r="I79" s="24" t="s">
         <v>367</v>
       </c>
       <c r="J79" s="19">
@@ -5830,10 +5833,10 @@
       <c r="G80" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H80" s="25" t="s">
+      <c r="H80" s="24" t="s">
         <v>370</v>
       </c>
-      <c r="I80" s="25" t="s">
+      <c r="I80" s="24" t="s">
         <v>371</v>
       </c>
       <c r="J80" s="19">
@@ -5865,10 +5868,10 @@
       <c r="G81" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H81" s="25" t="s">
+      <c r="H81" s="24" t="s">
         <v>375</v>
       </c>
-      <c r="I81" s="25" t="s">
+      <c r="I81" s="24" t="s">
         <v>376</v>
       </c>
       <c r="J81" s="19">
@@ -5900,10 +5903,10 @@
       <c r="G82" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H82" s="25" t="s">
+      <c r="H82" s="24" t="s">
         <v>380</v>
       </c>
-      <c r="I82" s="25" t="s">
+      <c r="I82" s="24" t="s">
         <v>381</v>
       </c>
       <c r="J82" s="19">
@@ -5935,10 +5938,10 @@
       <c r="G83" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H83" s="25" t="s">
+      <c r="H83" s="24" t="s">
         <v>384</v>
       </c>
-      <c r="I83" s="25" t="s">
+      <c r="I83" s="24" t="s">
         <v>385</v>
       </c>
       <c r="J83" s="19">
@@ -5970,10 +5973,10 @@
       <c r="G84" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H84" s="25" t="s">
+      <c r="H84" s="24" t="s">
         <v>388</v>
       </c>
-      <c r="I84" s="25" t="s">
+      <c r="I84" s="24" t="s">
         <v>389</v>
       </c>
       <c r="J84" s="19">
@@ -6005,10 +6008,10 @@
       <c r="G85" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H85" s="25" t="s">
+      <c r="H85" s="24" t="s">
         <v>394</v>
       </c>
-      <c r="I85" s="25" t="s">
+      <c r="I85" s="24" t="s">
         <v>395</v>
       </c>
       <c r="J85" s="19">
@@ -6040,10 +6043,10 @@
       <c r="G86" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H86" s="25" t="s">
+      <c r="H86" s="24" t="s">
         <v>398</v>
       </c>
-      <c r="I86" s="25" t="s">
+      <c r="I86" s="24" t="s">
         <v>399</v>
       </c>
       <c r="J86" s="19">
@@ -6075,10 +6078,10 @@
       <c r="G87" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H87" s="25" t="s">
+      <c r="H87" s="24" t="s">
         <v>402</v>
       </c>
-      <c r="I87" s="25" t="s">
+      <c r="I87" s="24" t="s">
         <v>403</v>
       </c>
       <c r="J87" s="19">
@@ -6110,10 +6113,10 @@
       <c r="G88" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H88" s="25" t="s">
+      <c r="H88" s="24" t="s">
         <v>407</v>
       </c>
-      <c r="I88" s="25" t="s">
+      <c r="I88" s="24" t="s">
         <v>408</v>
       </c>
       <c r="J88" s="19">
@@ -6145,10 +6148,10 @@
       <c r="G89" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H89" s="25" t="s">
+      <c r="H89" s="24" t="s">
         <v>411</v>
       </c>
-      <c r="I89" s="25" t="s">
+      <c r="I89" s="24" t="s">
         <v>412</v>
       </c>
       <c r="J89" s="19">
@@ -6180,10 +6183,10 @@
       <c r="G90" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H90" s="25" t="s">
+      <c r="H90" s="24" t="s">
         <v>415</v>
       </c>
-      <c r="I90" s="25" t="s">
+      <c r="I90" s="24" t="s">
         <v>416</v>
       </c>
       <c r="J90" s="19">
@@ -6215,10 +6218,10 @@
       <c r="G91" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H91" s="25" t="s">
+      <c r="H91" s="24" t="s">
         <v>419</v>
       </c>
-      <c r="I91" s="25" t="s">
+      <c r="I91" s="24" t="s">
         <v>420</v>
       </c>
       <c r="J91" s="19">
@@ -6250,10 +6253,10 @@
       <c r="G92" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H92" s="25" t="s">
+      <c r="H92" s="24" t="s">
         <v>423</v>
       </c>
-      <c r="I92" s="25" t="s">
+      <c r="I92" s="24" t="s">
         <v>424</v>
       </c>
       <c r="J92" s="19">
@@ -6285,10 +6288,10 @@
       <c r="G93" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H93" s="25" t="s">
+      <c r="H93" s="24" t="s">
         <v>427</v>
       </c>
-      <c r="I93" s="25" t="s">
+      <c r="I93" s="24" t="s">
         <v>428</v>
       </c>
       <c r="J93" s="19">
@@ -6320,10 +6323,10 @@
       <c r="G94" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H94" s="25" t="s">
+      <c r="H94" s="24" t="s">
         <v>431</v>
       </c>
-      <c r="I94" s="25" t="s">
+      <c r="I94" s="24" t="s">
         <v>432</v>
       </c>
       <c r="J94" s="19">
@@ -6355,10 +6358,10 @@
       <c r="G95" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H95" s="25" t="s">
+      <c r="H95" s="24" t="s">
         <v>435</v>
       </c>
-      <c r="I95" s="25" t="s">
+      <c r="I95" s="24" t="s">
         <v>436</v>
       </c>
       <c r="J95" s="19">
@@ -6390,10 +6393,10 @@
       <c r="G96" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H96" s="25" t="s">
+      <c r="H96" s="24" t="s">
         <v>440</v>
       </c>
-      <c r="I96" s="25" t="s">
+      <c r="I96" s="24" t="s">
         <v>441</v>
       </c>
       <c r="J96" s="19">
@@ -6425,10 +6428,10 @@
       <c r="G97" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H97" s="25" t="s">
+      <c r="H97" s="24" t="s">
         <v>444</v>
       </c>
-      <c r="I97" s="25" t="s">
+      <c r="I97" s="24" t="s">
         <v>445</v>
       </c>
       <c r="J97" s="19">
@@ -6460,10 +6463,10 @@
       <c r="G98" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H98" s="25" t="s">
+      <c r="H98" s="24" t="s">
         <v>448</v>
       </c>
-      <c r="I98" s="25" t="s">
+      <c r="I98" s="24" t="s">
         <v>449</v>
       </c>
       <c r="J98" s="19">
@@ -6495,10 +6498,10 @@
       <c r="G99" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H99" s="25" t="s">
+      <c r="H99" s="24" t="s">
         <v>452</v>
       </c>
-      <c r="I99" s="25" t="s">
+      <c r="I99" s="24" t="s">
         <v>453</v>
       </c>
       <c r="J99" s="19">
@@ -6530,10 +6533,10 @@
       <c r="G100" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H100" s="25" t="s">
+      <c r="H100" s="24" t="s">
         <v>457</v>
       </c>
-      <c r="I100" s="25" t="s">
+      <c r="I100" s="24" t="s">
         <v>458</v>
       </c>
       <c r="J100" s="19">
@@ -6565,10 +6568,10 @@
       <c r="G101" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H101" s="25" t="s">
+      <c r="H101" s="24" t="s">
         <v>461</v>
       </c>
-      <c r="I101" s="25" t="s">
+      <c r="I101" s="24" t="s">
         <v>462</v>
       </c>
       <c r="J101" s="19">
@@ -6600,10 +6603,10 @@
       <c r="G102" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H102" s="25" t="s">
+      <c r="H102" s="24" t="s">
         <v>465</v>
       </c>
-      <c r="I102" s="25" t="s">
+      <c r="I102" s="24" t="s">
         <v>466</v>
       </c>
       <c r="J102" s="19">
@@ -6635,10 +6638,10 @@
       <c r="G103" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H103" s="25" t="s">
+      <c r="H103" s="24" t="s">
         <v>469</v>
       </c>
-      <c r="I103" s="25" t="s">
+      <c r="I103" s="24" t="s">
         <v>470</v>
       </c>
       <c r="J103" s="19">
@@ -6670,10 +6673,10 @@
       <c r="G104" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H104" s="25" t="s">
+      <c r="H104" s="24" t="s">
         <v>473</v>
       </c>
-      <c r="I104" s="25" t="s">
+      <c r="I104" s="24" t="s">
         <v>474</v>
       </c>
       <c r="J104" s="19">
@@ -6705,10 +6708,10 @@
       <c r="G105" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H105" s="25" t="s">
+      <c r="H105" s="24" t="s">
         <v>478</v>
       </c>
-      <c r="I105" s="25" t="s">
+      <c r="I105" s="24" t="s">
         <v>479</v>
       </c>
       <c r="J105" s="19">
@@ -6740,10 +6743,10 @@
       <c r="G106" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H106" s="25" t="s">
+      <c r="H106" s="24" t="s">
         <v>482</v>
       </c>
-      <c r="I106" s="25" t="s">
+      <c r="I106" s="24" t="s">
         <v>483</v>
       </c>
       <c r="J106" s="19">
@@ -6775,10 +6778,10 @@
       <c r="G107" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H107" s="25" t="s">
+      <c r="H107" s="24" t="s">
         <v>487</v>
       </c>
-      <c r="I107" s="25" t="s">
+      <c r="I107" s="24" t="s">
         <v>488</v>
       </c>
       <c r="J107" s="19">
@@ -6810,10 +6813,10 @@
       <c r="G108" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H108" s="25" t="s">
+      <c r="H108" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="I108" s="25" t="s">
+      <c r="I108" s="24" t="s">
         <v>492</v>
       </c>
       <c r="J108" s="19">
@@ -6845,10 +6848,10 @@
       <c r="G109" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H109" s="25" t="s">
+      <c r="H109" s="24" t="s">
         <v>496</v>
       </c>
-      <c r="I109" s="25" t="s">
+      <c r="I109" s="24" t="s">
         <v>497</v>
       </c>
       <c r="J109" s="19">
@@ -6880,10 +6883,10 @@
       <c r="G110" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H110" s="25" t="s">
+      <c r="H110" s="24" t="s">
         <v>500</v>
       </c>
-      <c r="I110" s="25" t="s">
+      <c r="I110" s="24" t="s">
         <v>501</v>
       </c>
       <c r="J110" s="19">
@@ -6915,10 +6918,10 @@
       <c r="G111" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H111" s="25" t="s">
+      <c r="H111" s="24" t="s">
         <v>504</v>
       </c>
-      <c r="I111" s="25" t="s">
+      <c r="I111" s="24" t="s">
         <v>505</v>
       </c>
       <c r="J111" s="19">
@@ -6950,10 +6953,10 @@
       <c r="G112" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H112" s="25" t="s">
+      <c r="H112" s="24" t="s">
         <v>509</v>
       </c>
-      <c r="I112" s="25" t="s">
+      <c r="I112" s="24" t="s">
         <v>510</v>
       </c>
       <c r="J112" s="19">
@@ -6985,10 +6988,10 @@
       <c r="G113" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H113" s="25" t="s">
+      <c r="H113" s="24" t="s">
         <v>514</v>
       </c>
-      <c r="I113" s="25" t="s">
+      <c r="I113" s="24" t="s">
         <v>515</v>
       </c>
       <c r="J113" s="19">
@@ -7020,10 +7023,10 @@
       <c r="G114" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H114" s="25" t="s">
+      <c r="H114" s="24" t="s">
         <v>518</v>
       </c>
-      <c r="I114" s="25" t="s">
+      <c r="I114" s="24" t="s">
         <v>519</v>
       </c>
       <c r="J114" s="19">
@@ -7055,10 +7058,10 @@
       <c r="G115" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H115" s="25" t="s">
+      <c r="H115" s="24" t="s">
         <v>522</v>
       </c>
-      <c r="I115" s="25" t="s">
+      <c r="I115" s="24" t="s">
         <v>523</v>
       </c>
       <c r="J115" s="19">
@@ -7090,10 +7093,10 @@
       <c r="G116" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H116" s="25" t="s">
+      <c r="H116" s="24" t="s">
         <v>526</v>
       </c>
-      <c r="I116" s="25" t="s">
+      <c r="I116" s="24" t="s">
         <v>527</v>
       </c>
       <c r="J116" s="19">
@@ -7125,10 +7128,10 @@
       <c r="G117" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H117" s="25" t="s">
+      <c r="H117" s="24" t="s">
         <v>531</v>
       </c>
-      <c r="I117" s="25" t="s">
+      <c r="I117" s="24" t="s">
         <v>532</v>
       </c>
       <c r="J117" s="19">
@@ -7160,10 +7163,10 @@
       <c r="G118" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H118" s="25" t="s">
+      <c r="H118" s="24" t="s">
         <v>535</v>
       </c>
-      <c r="I118" s="25" t="s">
+      <c r="I118" s="24" t="s">
         <v>536</v>
       </c>
       <c r="J118" s="19">
@@ -7195,10 +7198,10 @@
       <c r="G119" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H119" s="25" t="s">
+      <c r="H119" s="24" t="s">
         <v>541</v>
       </c>
-      <c r="I119" s="25" t="s">
+      <c r="I119" s="24" t="s">
         <v>542</v>
       </c>
       <c r="J119" s="19">
@@ -7230,10 +7233,10 @@
       <c r="G120" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H120" s="25" t="s">
+      <c r="H120" s="24" t="s">
         <v>546</v>
       </c>
-      <c r="I120" s="25" t="s">
+      <c r="I120" s="24" t="s">
         <v>547</v>
       </c>
       <c r="J120" s="19">
@@ -7265,10 +7268,10 @@
       <c r="G121" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H121" s="25" t="s">
+      <c r="H121" s="24" t="s">
         <v>550</v>
       </c>
-      <c r="I121" s="25" t="s">
+      <c r="I121" s="24" t="s">
         <v>551</v>
       </c>
       <c r="J121" s="19">
@@ -7300,10 +7303,10 @@
       <c r="G122" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H122" s="25" t="s">
+      <c r="H122" s="24" t="s">
         <v>555</v>
       </c>
-      <c r="I122" s="25" t="s">
+      <c r="I122" s="24" t="s">
         <v>556</v>
       </c>
       <c r="J122" s="19">
@@ -7335,10 +7338,10 @@
       <c r="G123" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H123" s="25" t="s">
+      <c r="H123" s="24" t="s">
         <v>560</v>
       </c>
-      <c r="I123" s="25" t="s">
+      <c r="I123" s="24" t="s">
         <v>561</v>
       </c>
       <c r="J123" s="19">
@@ -7370,10 +7373,10 @@
       <c r="G124" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H124" s="25" t="s">
+      <c r="H124" s="24" t="s">
         <v>564</v>
       </c>
-      <c r="I124" s="25" t="s">
+      <c r="I124" s="24" t="s">
         <v>565</v>
       </c>
       <c r="J124" s="19">
@@ -7405,10 +7408,10 @@
       <c r="G125" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H125" s="25" t="s">
+      <c r="H125" s="24" t="s">
         <v>569</v>
       </c>
-      <c r="I125" s="25" t="s">
+      <c r="I125" s="24" t="s">
         <v>570</v>
       </c>
       <c r="J125" s="19">
@@ -7440,10 +7443,10 @@
       <c r="G126" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H126" s="25" t="s">
+      <c r="H126" s="24" t="s">
         <v>573</v>
       </c>
-      <c r="I126" s="25" t="s">
+      <c r="I126" s="24" t="s">
         <v>574</v>
       </c>
       <c r="J126" s="19">
@@ -7475,10 +7478,10 @@
       <c r="G127" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H127" s="25" t="s">
+      <c r="H127" s="24" t="s">
         <v>578</v>
       </c>
-      <c r="I127" s="25" t="s">
+      <c r="I127" s="24" t="s">
         <v>579</v>
       </c>
       <c r="J127" s="19">
@@ -7510,10 +7513,10 @@
       <c r="G128" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H128" s="25" t="s">
+      <c r="H128" s="24" t="s">
         <v>582</v>
       </c>
-      <c r="I128" s="25" t="s">
+      <c r="I128" s="24" t="s">
         <v>583</v>
       </c>
       <c r="J128" s="19">
@@ -7545,10 +7548,10 @@
       <c r="G129" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H129" s="25" t="s">
+      <c r="H129" s="24" t="s">
         <v>589</v>
       </c>
-      <c r="I129" s="25" t="s">
+      <c r="I129" s="24" t="s">
         <v>590</v>
       </c>
       <c r="J129" s="19">
@@ -7580,10 +7583,10 @@
       <c r="G130" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H130" s="25" t="s">
+      <c r="H130" s="24" t="s">
         <v>593</v>
       </c>
-      <c r="I130" s="25" t="s">
+      <c r="I130" s="24" t="s">
         <v>594</v>
       </c>
       <c r="J130" s="19">
@@ -7615,10 +7618,10 @@
       <c r="G131" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H131" s="25" t="s">
+      <c r="H131" s="24" t="s">
         <v>598</v>
       </c>
-      <c r="I131" s="25" t="s">
+      <c r="I131" s="24" t="s">
         <v>599</v>
       </c>
       <c r="J131" s="19">
@@ -7650,10 +7653,10 @@
       <c r="G132" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H132" s="25" t="s">
+      <c r="H132" s="24" t="s">
         <v>603</v>
       </c>
-      <c r="I132" s="25" t="s">
+      <c r="I132" s="24" t="s">
         <v>604</v>
       </c>
       <c r="J132" s="19">
@@ -7685,10 +7688,10 @@
       <c r="G133" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H133" s="25" t="s">
+      <c r="H133" s="24" t="s">
         <v>607</v>
       </c>
-      <c r="I133" s="25" t="s">
+      <c r="I133" s="24" t="s">
         <v>608</v>
       </c>
       <c r="J133" s="19">
@@ -7720,10 +7723,10 @@
       <c r="G134" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H134" s="25" t="s">
+      <c r="H134" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="I134" s="25" t="s">
+      <c r="I134" s="24" t="s">
         <v>612</v>
       </c>
       <c r="J134" s="19">
@@ -7755,10 +7758,10 @@
       <c r="G135" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H135" s="25" t="s">
+      <c r="H135" s="24" t="s">
         <v>615</v>
       </c>
-      <c r="I135" s="25" t="s">
+      <c r="I135" s="24" t="s">
         <v>616</v>
       </c>
       <c r="J135" s="19">
@@ -7790,10 +7793,10 @@
       <c r="G136" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H136" s="25" t="s">
+      <c r="H136" s="24" t="s">
         <v>619</v>
       </c>
-      <c r="I136" s="25" t="s">
+      <c r="I136" s="24" t="s">
         <v>620</v>
       </c>
       <c r="J136" s="19">
@@ -7825,10 +7828,10 @@
       <c r="G137" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="H137" s="25" t="s">
+      <c r="H137" s="24" t="s">
         <v>623</v>
       </c>
-      <c r="I137" s="25" t="s">
+      <c r="I137" s="24" t="s">
         <v>624</v>
       </c>
       <c r="J137" s="19">
@@ -7860,10 +7863,10 @@
       <c r="G138" s="19" t="s">
         <v>627</v>
       </c>
-      <c r="H138" s="25" t="s">
+      <c r="H138" s="24" t="s">
         <v>628</v>
       </c>
-      <c r="I138" s="25" t="s">
+      <c r="I138" s="24" t="s">
         <v>629</v>
       </c>
       <c r="J138" s="19">
@@ -7895,10 +7898,10 @@
       <c r="G139" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H139" s="25" t="s">
+      <c r="H139" s="24" t="s">
         <v>632</v>
       </c>
-      <c r="I139" s="25" t="s">
+      <c r="I139" s="24" t="s">
         <v>633</v>
       </c>
       <c r="J139" s="19">
@@ -7930,10 +7933,10 @@
       <c r="G140" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H140" s="25" t="s">
+      <c r="H140" s="24" t="s">
         <v>638</v>
       </c>
-      <c r="I140" s="25" t="s">
+      <c r="I140" s="24" t="s">
         <v>639</v>
       </c>
       <c r="J140" s="19">
@@ -7965,10 +7968,10 @@
       <c r="G141" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H141" s="25" t="s">
+      <c r="H141" s="24" t="s">
         <v>642</v>
       </c>
-      <c r="I141" s="25" t="s">
+      <c r="I141" s="24" t="s">
         <v>643</v>
       </c>
       <c r="J141" s="19">
@@ -8000,10 +8003,10 @@
       <c r="G142" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H142" s="25" t="s">
+      <c r="H142" s="24" t="s">
         <v>646</v>
       </c>
-      <c r="I142" s="25" t="s">
+      <c r="I142" s="24" t="s">
         <v>647</v>
       </c>
       <c r="J142" s="19">
@@ -8035,10 +8038,10 @@
       <c r="G143" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H143" s="25" t="s">
+      <c r="H143" s="24" t="s">
         <v>651</v>
       </c>
-      <c r="I143" s="25" t="s">
+      <c r="I143" s="24" t="s">
         <v>652</v>
       </c>
       <c r="J143" s="19">
@@ -8070,10 +8073,10 @@
       <c r="G144" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H144" s="25" t="s">
+      <c r="H144" s="24" t="s">
         <v>655</v>
       </c>
-      <c r="I144" s="25" t="s">
+      <c r="I144" s="24" t="s">
         <v>656</v>
       </c>
       <c r="J144" s="19">
@@ -8105,10 +8108,10 @@
       <c r="G145" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H145" s="25" t="s">
+      <c r="H145" s="24" t="s">
         <v>660</v>
       </c>
-      <c r="I145" s="25" t="s">
+      <c r="I145" s="24" t="s">
         <v>661</v>
       </c>
       <c r="J145" s="19">
@@ -8140,10 +8143,10 @@
       <c r="G146" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H146" s="25" t="s">
+      <c r="H146" s="24" t="s">
         <v>664</v>
       </c>
-      <c r="I146" s="25" t="s">
+      <c r="I146" s="24" t="s">
         <v>665</v>
       </c>
       <c r="J146" s="19">
@@ -8175,10 +8178,10 @@
       <c r="G147" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H147" s="25" t="s">
+      <c r="H147" s="24" t="s">
         <v>669</v>
       </c>
-      <c r="I147" s="25" t="s">
+      <c r="I147" s="24" t="s">
         <v>670</v>
       </c>
       <c r="J147" s="19">
@@ -8210,10 +8213,10 @@
       <c r="G148" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H148" s="25" t="s">
+      <c r="H148" s="24" t="s">
         <v>673</v>
       </c>
-      <c r="I148" s="25" t="s">
+      <c r="I148" s="24" t="s">
         <v>674</v>
       </c>
       <c r="J148" s="19">
@@ -8245,10 +8248,10 @@
       <c r="G149" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H149" s="25" t="s">
+      <c r="H149" s="24" t="s">
         <v>677</v>
       </c>
-      <c r="I149" s="25" t="s">
+      <c r="I149" s="24" t="s">
         <v>678</v>
       </c>
       <c r="J149" s="19">
@@ -8280,10 +8283,10 @@
       <c r="G150" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H150" s="25" t="s">
+      <c r="H150" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="I150" s="25" t="s">
+      <c r="I150" s="24" t="s">
         <v>682</v>
       </c>
       <c r="J150" s="19">
@@ -8315,10 +8318,10 @@
       <c r="G151" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H151" s="25" t="s">
+      <c r="H151" s="24" t="s">
         <v>685</v>
       </c>
-      <c r="I151" s="25" t="s">
+      <c r="I151" s="24" t="s">
         <v>686</v>
       </c>
       <c r="J151" s="19">
@@ -8350,10 +8353,10 @@
       <c r="G152" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H152" s="25" t="s">
+      <c r="H152" s="24" t="s">
         <v>692</v>
       </c>
-      <c r="I152" s="25" t="s">
+      <c r="I152" s="24" t="s">
         <v>693</v>
       </c>
       <c r="J152" s="19">
@@ -8385,10 +8388,10 @@
       <c r="G153" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H153" s="25" t="s">
+      <c r="H153" s="24" t="s">
         <v>696</v>
       </c>
-      <c r="I153" s="25" t="s">
+      <c r="I153" s="24" t="s">
         <v>697</v>
       </c>
       <c r="J153" s="19">
@@ -8420,10 +8423,10 @@
       <c r="G154" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H154" s="25" t="s">
+      <c r="H154" s="24" t="s">
         <v>701</v>
       </c>
-      <c r="I154" s="25" t="s">
+      <c r="I154" s="24" t="s">
         <v>702</v>
       </c>
       <c r="J154" s="19">
@@ -8455,10 +8458,10 @@
       <c r="G155" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H155" s="25" t="s">
+      <c r="H155" s="24" t="s">
         <v>706</v>
       </c>
-      <c r="I155" s="25" t="s">
+      <c r="I155" s="24" t="s">
         <v>707</v>
       </c>
       <c r="J155" s="19">
@@ -8490,10 +8493,10 @@
       <c r="G156" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H156" s="25" t="s">
+      <c r="H156" s="24" t="s">
         <v>710</v>
       </c>
-      <c r="I156" s="25" t="s">
+      <c r="I156" s="24" t="s">
         <v>711</v>
       </c>
       <c r="J156" s="19">
@@ -8525,10 +8528,10 @@
       <c r="G157" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H157" s="25" t="s">
+      <c r="H157" s="24" t="s">
         <v>715</v>
       </c>
-      <c r="I157" s="25" t="s">
+      <c r="I157" s="24" t="s">
         <v>716</v>
       </c>
       <c r="J157" s="19">
@@ -8560,10 +8563,10 @@
       <c r="G158" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H158" s="25" t="s">
+      <c r="H158" s="24" t="s">
         <v>720</v>
       </c>
-      <c r="I158" s="25" t="s">
+      <c r="I158" s="24" t="s">
         <v>721</v>
       </c>
       <c r="J158" s="19">
@@ -8595,10 +8598,10 @@
       <c r="G159" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H159" s="25" t="s">
+      <c r="H159" s="24" t="s">
         <v>724</v>
       </c>
-      <c r="I159" s="25" t="s">
+      <c r="I159" s="24" t="s">
         <v>725</v>
       </c>
       <c r="J159" s="19">
@@ -8630,10 +8633,10 @@
       <c r="G160" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H160" s="25" t="s">
+      <c r="H160" s="24" t="s">
         <v>730</v>
       </c>
-      <c r="I160" s="25" t="s">
+      <c r="I160" s="24" t="s">
         <v>731</v>
       </c>
       <c r="J160" s="19">
@@ -8665,10 +8668,10 @@
       <c r="G161" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H161" s="25" t="s">
+      <c r="H161" s="24" t="s">
         <v>735</v>
       </c>
-      <c r="I161" s="25" t="s">
+      <c r="I161" s="24" t="s">
         <v>736</v>
       </c>
       <c r="J161" s="19">
@@ -8700,10 +8703,10 @@
       <c r="G162" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H162" s="25" t="s">
+      <c r="H162" s="24" t="s">
         <v>739</v>
       </c>
-      <c r="I162" s="25" t="s">
+      <c r="I162" s="24" t="s">
         <v>740</v>
       </c>
       <c r="J162" s="19">
@@ -8735,10 +8738,10 @@
       <c r="G163" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H163" s="25" t="s">
+      <c r="H163" s="24" t="s">
         <v>743</v>
       </c>
-      <c r="I163" s="25" t="s">
+      <c r="I163" s="24" t="s">
         <v>744</v>
       </c>
       <c r="J163" s="19">
@@ -8770,10 +8773,10 @@
       <c r="G164" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H164" s="25" t="s">
+      <c r="H164" s="24" t="s">
         <v>747</v>
       </c>
-      <c r="I164" s="25" t="s">
+      <c r="I164" s="24" t="s">
         <v>748</v>
       </c>
       <c r="J164" s="19">
@@ -8805,10 +8808,10 @@
       <c r="G165" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H165" s="25" t="s">
+      <c r="H165" s="24" t="s">
         <v>752</v>
       </c>
-      <c r="I165" s="25" t="s">
+      <c r="I165" s="24" t="s">
         <v>753</v>
       </c>
       <c r="J165" s="19">
@@ -8840,10 +8843,10 @@
       <c r="G166" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H166" s="25" t="s">
+      <c r="H166" s="24" t="s">
         <v>757</v>
       </c>
-      <c r="I166" s="25" t="s">
+      <c r="I166" s="24" t="s">
         <v>758</v>
       </c>
       <c r="J166" s="19">
@@ -8875,10 +8878,10 @@
       <c r="G167" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="H167" s="25" t="s">
+      <c r="H167" s="24" t="s">
         <v>761</v>
       </c>
-      <c r="I167" s="25" t="s">
+      <c r="I167" s="24" t="s">
         <v>762</v>
       </c>
       <c r="J167" s="19">
@@ -8910,10 +8913,10 @@
       <c r="G168" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H168" s="25" t="s">
+      <c r="H168" s="24" t="s">
         <v>765</v>
       </c>
-      <c r="I168" s="25" t="s">
+      <c r="I168" s="24" t="s">
         <v>766</v>
       </c>
       <c r="J168" s="19">

</xml_diff>

<commit_message>
T-027: 104-row coverage ledger; implementation complete, acceptance blocked on matrix and generator coverage
</commit_message>
<xml_diff>
--- a/Documentation/docs/Product Book/PPIQ_Backlog_v2_9_1_03Aug2026.xlsx
+++ b/Documentation/docs/Product Book/PPIQ_Backlog_v2_9_1_03Aug2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\PlantProcess-IQ\Documentation\docs\Product Book\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EB4BBDE-2C52-44DD-843B-BD99CB96710D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A65A5655-3E98-4654-8388-792E022B6792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="394" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="Legend" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$K$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$K$168</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -3992,38 +3992,38 @@
       </c>
     </row>
     <row r="28" spans="1:11" ht="75" x14ac:dyDescent="0.25">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="B28" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28" s="19" t="s">
+      <c r="B28" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="D28" s="19" t="s">
+      <c r="D28" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="E28" s="19" t="s">
+      <c r="E28" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="F28" s="19" t="s">
+      <c r="F28" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="G28" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="H28" s="24" t="s">
+      <c r="G28" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H28" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="I28" s="24" t="s">
+      <c r="I28" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="J28" s="19">
+      <c r="J28" s="18">
         <v>6</v>
       </c>
-      <c r="K28" s="19" t="s">
-        <v>90</v>
+      <c r="K28" s="18" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="45" x14ac:dyDescent="0.25">
@@ -4272,38 +4272,38 @@
       </c>
     </row>
     <row r="36" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A36" s="19" t="s">
+      <c r="A36" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="B36" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C36" s="19" t="s">
+      <c r="B36" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C36" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="D36" s="19" t="s">
+      <c r="D36" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="E36" s="19" t="s">
+      <c r="E36" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F36" s="19" t="s">
+      <c r="F36" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="G36" s="19" t="s">
+      <c r="G36" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="H36" s="24" t="s">
+      <c r="H36" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="I36" s="24" t="s">
+      <c r="I36" s="23" t="s">
         <v>178</v>
       </c>
-      <c r="J36" s="19">
+      <c r="J36" s="18">
         <v>8</v>
       </c>
-      <c r="K36" s="19" t="s">
-        <v>90</v>
+      <c r="K36" s="20" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="45" x14ac:dyDescent="0.25">
@@ -8927,7 +8927,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K165" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:K168" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
T-031 core implementation complete: Fleet-v2 donor alignment, staging regeneration, cross-layer certification GREEN with proven divergence
</commit_message>
<xml_diff>
--- a/Documentation/docs/Product Book/PPIQ_Backlog_v2_9_1_03Aug2026.xlsx
+++ b/Documentation/docs/Product Book/PPIQ_Backlog_v2_9_1_03Aug2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\PlantProcess-IQ\Documentation\docs\Product Book\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{709F8AA2-33D5-49F0-A186-E84E25CF4558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D2718D-834A-4088-9A41-0400A156476E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="394" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="394" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1788" uniqueCount="830">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1792" uniqueCount="834">
   <si>
     <t>Task Id</t>
   </si>
@@ -2529,12 +2529,27 @@
   </si>
   <si>
     <t>InProgress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total required till Presentation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total done </t>
+  </si>
+  <si>
+    <t>Total remaining</t>
+  </si>
+  <si>
+    <t>Percentage of done</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2667,7 +2682,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2740,6 +2755,15 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4355,73 +4379,73 @@
       </c>
     </row>
     <row r="38" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A38" s="19" t="s">
+      <c r="A38" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="B38" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C38" s="19" t="s">
+      <c r="B38" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="D38" s="19" t="s">
+      <c r="D38" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="E38" s="19" t="s">
+      <c r="E38" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F38" s="19" t="s">
+      <c r="F38" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="G38" s="19" t="s">
+      <c r="G38" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="H38" s="24" t="s">
+      <c r="H38" s="23" t="s">
         <v>185</v>
       </c>
-      <c r="I38" s="24" t="s">
+      <c r="I38" s="23" t="s">
         <v>186</v>
       </c>
-      <c r="J38" s="19">
+      <c r="J38" s="18">
         <v>3</v>
       </c>
-      <c r="K38" s="19" t="s">
-        <v>90</v>
+      <c r="K38" s="20" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A39" s="19" t="s">
+      <c r="A39" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="B39" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C39" s="19" t="s">
+      <c r="B39" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="D39" s="19" t="s">
+      <c r="D39" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="E39" s="19" t="s">
+      <c r="E39" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F39" s="19" t="s">
+      <c r="F39" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="G39" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="H39" s="24" t="s">
+      <c r="G39" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H39" s="23" t="s">
         <v>189</v>
       </c>
-      <c r="I39" s="24" t="s">
+      <c r="I39" s="23" t="s">
         <v>190</v>
       </c>
-      <c r="J39" s="19">
-        <v>12</v>
-      </c>
-      <c r="K39" s="19" t="s">
-        <v>90</v>
+      <c r="J39" s="18">
+        <v>12</v>
+      </c>
+      <c r="K39" s="20" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="60" x14ac:dyDescent="0.25">
@@ -8947,7 +8971,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -8956,9 +8980,11 @@
     <col min="4" max="4" width="80" customWidth="1"/>
     <col min="5" max="5" width="8" customWidth="1"/>
     <col min="6" max="6" width="9" customWidth="1"/>
+    <col min="7" max="7" width="12.5703125" customWidth="1"/>
+    <col min="8" max="8" width="26.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -8978,7 +9004,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
@@ -9000,7 +9026,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>81</v>
       </c>
@@ -9022,7 +9048,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>153</v>
       </c>
@@ -9043,8 +9069,15 @@
         <f>SUMIF(Backlog!C:C,A4,Backlog!J:J)</f>
         <v>107</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H4" s="31" t="s">
+        <v>830</v>
+      </c>
+      <c r="I4" s="32">
+        <f>SUM(F2:F7)</f>
+        <v>574</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>201</v>
       </c>
@@ -9065,8 +9098,14 @@
         <f>SUMIF(Backlog!C:C,A5,Backlog!J:J)</f>
         <v>80</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H5" s="32" t="s">
+        <v>831</v>
+      </c>
+      <c r="I5" s="32">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>251</v>
       </c>
@@ -9087,8 +9126,15 @@
         <f>SUMIF(Backlog!C:C,A6,Backlog!J:J)</f>
         <v>106</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H6" s="32" t="s">
+        <v>832</v>
+      </c>
+      <c r="I6" s="32">
+        <f>I4-I5</f>
+        <v>289</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>322</v>
       </c>
@@ -9109,8 +9155,15 @@
         <f>SUMIF(Backlog!C:C,A7,Backlog!J:J)</f>
         <v>83</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H7" s="32" t="s">
+        <v>833</v>
+      </c>
+      <c r="I7" s="33">
+        <f>(I5/I4)</f>
+        <v>0.49651567944250868</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>392</v>
       </c>
@@ -9132,7 +9185,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>438</v>
       </c>
@@ -9154,7 +9207,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>485</v>
       </c>
@@ -9176,7 +9229,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>538</v>
       </c>
@@ -9198,7 +9251,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>586</v>
       </c>
@@ -9220,7 +9273,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>635</v>
       </c>
@@ -9242,7 +9295,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>689</v>
       </c>
@@ -9264,7 +9317,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>727</v>
       </c>
@@ -9286,7 +9339,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C16" s="7" t="s">
         <v>799</v>
       </c>

</xml_diff>